<commit_message>
RC task: drop the 5-step start charge, 15 steps per error; bonus targets 25/70/55/55 from the simulations
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/task/RC/Resources/PigeonTaskConditions.xlsx
+++ b/task/RC/Resources/PigeonTaskConditions.xlsx
@@ -514,13 +514,13 @@
         <v>1000</v>
       </c>
       <c r="F2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H2" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -567,13 +567,13 @@
         <v>1000</v>
       </c>
       <c r="F3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H3" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -620,13 +620,13 @@
         <v>1000</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H4" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I4" t="n">
         <v>0</v>
@@ -673,13 +673,13 @@
         <v>1000</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H5" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>

</xml_diff>